<commit_message>
Use exact Opella reported revenue
</commit_message>
<xml_diff>
--- a/public/downloads/opella/Opella-Carveout-Model.xlsx
+++ b/public/downloads/opella/Opella-Carveout-Model.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abbah\Downloads\Portefolio\Portefolio\Sidetrade\public\downloads\opella\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abbah\AppData\Local\Temp\OP-FIN-EXACT-REVENUE-02-20260812\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D6DF02F5-A45C-4D06-B4E7-EC6FD1B45366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8B6BDEF-80D4-4BB2-A4EC-91701E0F145B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-300" yWindow="6630" windowWidth="28800" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -426,31 +426,31 @@
     <t>M1 — Périmètre et ancrages</t>
   </si>
   <si>
-    <t>Chiffre d'affaires FY2024 arrondi retenu par le modèle (M€)</t>
+    <t>Chiffre d'affaires FY2024 publié retenu par le modèle (M€)</t>
+  </si>
+  <si>
+    <t>public</t>
+  </si>
+  <si>
+    <t>CA de 4 948 M€ publié par Sanofi selon son nouveau périmètre de reporting</t>
+  </si>
+  <si>
+    <t>Chiffre d'affaires FY2024 publié par Sanofi (M€)</t>
+  </si>
+  <si>
+    <t>résultats FY2024 Sanofi, p. 10, nouveau périmètre de reporting</t>
+  </si>
+  <si>
+    <t>Marge d'EBITDA implicite du modèle</t>
   </si>
   <si>
     <t>calculé</t>
   </si>
   <si>
-    <t>arrondi à la Md€ la plus proche du CA de 4 948 M€ publié par Sanofi selon son nouveau périmètre de reporting</t>
-  </si>
-  <si>
-    <t>Chiffre d'affaires FY2024 publié par Sanofi (M€)</t>
-  </si>
-  <si>
-    <t>public</t>
-  </si>
-  <si>
-    <t>résultats FY2024 Sanofi, p. 10, nouveau périmètre de reporting</t>
-  </si>
-  <si>
-    <t>Marge d'EBITDA implicite du modèle</t>
-  </si>
-  <si>
     <t>S1+S5</t>
   </si>
   <si>
-    <t>proxy EBITDA implicite ÷ CA arrondi du modèle ; cette marge n'est pas publiée</t>
+    <t>proxy EBITDA implicite ÷ CA FY2024 publié ; cette marge n'est pas publiée</t>
   </si>
   <si>
     <t>EBITDA 2024E implicite de transaction (M€)</t>
@@ -1453,7 +1453,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1474,11 +1474,12 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2114,7 +2115,7 @@
       </c>
     </row>
     <row r="3" spans="2:8" ht="72" x14ac:dyDescent="0.25">
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>405</v>
       </c>
     </row>
@@ -2155,7 +2156,7 @@
         <v>295.7</v>
       </c>
       <c r="F6" s="15">
-        <v>252.32809000000009</v>
+        <v>253.46219086400001</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>86</v>
@@ -2176,7 +2177,7 @@
         <v>295.7</v>
       </c>
       <c r="F7" s="15">
-        <v>321.37667520000008</v>
+        <v>323.21991217792021</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>91</v>
@@ -2197,7 +2198,7 @@
         <v>295.7</v>
       </c>
       <c r="F8" s="15">
-        <v>434.58572321967989</v>
+        <v>437.91169289819538</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>101</v>
@@ -2220,7 +2221,7 @@
         <v>280.7</v>
       </c>
       <c r="F10" s="15">
-        <v>309.67667519999998</v>
+        <v>311.51991217792011</v>
       </c>
       <c r="G10" s="6" t="s">
         <v>91</v>
@@ -2241,7 +2242,7 @@
         <v>295.7</v>
       </c>
       <c r="F11" s="15">
-        <v>321.37667520000008</v>
+        <v>323.21991217792021</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>91</v>
@@ -2262,7 +2263,7 @@
         <v>349.7</v>
       </c>
       <c r="F12" s="15">
-        <v>377.21735991627048</v>
+        <v>381.31822177314132</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>418</v>
@@ -2285,7 +2286,7 @@
         <v>257.7</v>
       </c>
       <c r="F14" s="15">
-        <v>291.73667520000009</v>
+        <v>293.57991217792011</v>
       </c>
       <c r="G14" s="6" t="s">
         <v>91</v>
@@ -2306,7 +2307,7 @@
         <v>295.7</v>
       </c>
       <c r="F15" s="15">
-        <v>321.37667520000008</v>
+        <v>323.21991217792021</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>91</v>
@@ -2327,7 +2328,7 @@
         <v>364.1</v>
       </c>
       <c r="F16" s="15">
-        <v>374.72867520000011</v>
+        <v>376.57191217792013</v>
       </c>
       <c r="G16" s="6" t="s">
         <v>91</v>
@@ -2350,7 +2351,7 @@
         <v>295.7</v>
       </c>
       <c r="F18" s="15">
-        <v>335.3332602497602</v>
+        <v>338.45822874316241</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>101</v>
@@ -2371,7 +2372,7 @@
         <v>295.7</v>
       </c>
       <c r="F19" s="15">
-        <v>321.37667520000008</v>
+        <v>323.21991217792021</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>91</v>
@@ -2392,7 +2393,7 @@
         <v>295.7</v>
       </c>
       <c r="F20" s="15">
-        <v>313.89920000000012</v>
+        <v>315.82020272000011</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>91</v>
@@ -2423,7 +2424,7 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="48" x14ac:dyDescent="0.25">
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>422</v>
       </c>
     </row>
@@ -2431,7 +2432,7 @@
       <c r="B5" s="6" t="s">
         <v>423</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="32">
         <v>4</v>
       </c>
       <c r="D5" s="13" t="s">
@@ -2442,9 +2443,9 @@
       <c r="B6" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="23">
         <f>'M6 Bridge'!C33</f>
-        <v>1384.7377484414001</v>
+        <v>1382.7033880515855</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.25">
@@ -2453,25 +2454,25 @@
       </c>
       <c r="C7" s="15">
         <f>'M8 Acquéreur'!C5*'M8 Acquéreur'!C6</f>
-        <v>5538.9509937656003</v>
+        <v>5530.8135522063421</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>427</v>
       </c>
-      <c r="C8" s="20">
+      <c r="C8" s="21">
         <f>Hypothèses!C10-'M8 Acquéreur'!C7</f>
-        <v>10461.0490062344</v>
+        <v>10469.186447793658</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="22.5" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>428</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="23">
         <f>'M7 Financement'!C71</f>
-        <v>321.37667520000002</v>
+        <v>323.21991217792032</v>
       </c>
       <c r="D10" s="13" t="s">
         <v>429</v>
@@ -2903,12 +2904,12 @@
         <v>126</v>
       </c>
     </row>
-    <row r="6" spans="2:6" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
         <v>127</v>
       </c>
       <c r="C6" s="12">
-        <v>5000</v>
+        <v>4948</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>128</v>
@@ -2928,24 +2929,25 @@
         <v>4948</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E7" s="8" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="C8" s="14">
+        <f>C9/C6</f>
+        <v>0.23097355352812105</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>133</v>
-      </c>
-      <c r="C8" s="14">
-        <v>0.2286</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>128</v>
       </c>
       <c r="E8" s="8" t="s">
         <v>134</v>
@@ -2959,11 +2961,11 @@
         <v>136</v>
       </c>
       <c r="C9" s="15">
-        <f>C6*C8</f>
-        <v>1143</v>
+        <f>C10/14</f>
+        <v>1142.8571428571429</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="E9" s="8" t="s">
         <v>19</v>
@@ -2980,7 +2982,7 @@
         <v>16000</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>19</v>
@@ -2995,10 +2997,10 @@
       </c>
       <c r="C11" s="16">
         <f>C10/C9</f>
-        <v>13.99825021872266</v>
+        <v>14</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>19</v>
@@ -3015,7 +3017,7 @@
         <v>0.5</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>21</v>
@@ -3032,7 +3034,7 @@
         <v>0.48199999999999998</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>21</v>
@@ -3049,7 +3051,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>21</v>
@@ -3067,7 +3069,7 @@
         <v>1</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>21</v>
@@ -3124,7 +3126,7 @@
       <c r="B22" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="19">
         <v>1.6E-2</v>
       </c>
       <c r="D22" s="8" t="s">
@@ -3249,7 +3251,7 @@
       </c>
     </row>
     <row r="3" spans="2:10" ht="36" x14ac:dyDescent="0.25">
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>170</v>
       </c>
     </row>
@@ -3522,31 +3524,31 @@
       <c r="B15" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="C15" s="20">
+      <c r="C15" s="21">
         <f t="shared" ref="C15:I15" si="1">SUM(C11:C14)</f>
         <v>-120</v>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="21">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E15" s="20">
+      <c r="E15" s="21">
         <f t="shared" si="1"/>
         <v>-45.75</v>
       </c>
-      <c r="F15" s="20">
+      <c r="F15" s="21">
         <f t="shared" si="1"/>
         <v>-101</v>
       </c>
-      <c r="G15" s="20">
+      <c r="G15" s="21">
         <f t="shared" si="1"/>
         <v>-120</v>
       </c>
-      <c r="H15" s="20">
+      <c r="H15" s="21">
         <f t="shared" si="1"/>
         <v>-120</v>
       </c>
-      <c r="I15" s="20">
+      <c r="I15" s="21">
         <f t="shared" si="1"/>
         <v>-120</v>
       </c>
@@ -3572,7 +3574,7 @@
       </c>
     </row>
     <row r="3" spans="2:15" ht="48" x14ac:dyDescent="0.25">
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>188</v>
       </c>
     </row>
@@ -3624,7 +3626,7 @@
       <c r="B6" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="22">
         <v>-2.1</v>
       </c>
       <c r="D6" s="7">
@@ -3670,7 +3672,7 @@
       <c r="B7" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="C7" s="21">
+      <c r="C7" s="22">
         <v>-1.25</v>
       </c>
       <c r="D7" s="7">
@@ -3716,7 +3718,7 @@
       <c r="B8" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="22">
         <v>-0.85</v>
       </c>
       <c r="D8" s="7">
@@ -3762,7 +3764,7 @@
       <c r="B9" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="21">
+      <c r="C9" s="22">
         <v>-0.5</v>
       </c>
       <c r="D9" s="7">
@@ -3808,7 +3810,7 @@
       <c r="B10" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="C10" s="21">
+      <c r="C10" s="22">
         <v>-0.3</v>
       </c>
       <c r="D10" s="7">
@@ -3854,27 +3856,27 @@
       <c r="B11" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="I11" s="20">
+      <c r="I11" s="21">
         <f t="shared" ref="I11:N11" si="0">SUM(I6:I10)</f>
         <v>0</v>
       </c>
-      <c r="J11" s="20">
+      <c r="J11" s="21">
         <f t="shared" si="0"/>
         <v>-40</v>
       </c>
-      <c r="K11" s="20">
+      <c r="K11" s="21">
         <f t="shared" si="0"/>
         <v>-48.300000000000011</v>
       </c>
-      <c r="L11" s="20">
+      <c r="L11" s="21">
         <f t="shared" si="0"/>
         <v>-10.4</v>
       </c>
-      <c r="M11" s="20">
+      <c r="M11" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N11" s="20">
+      <c r="N11" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -3901,7 +3903,7 @@
       </c>
     </row>
     <row r="3" spans="2:10" ht="24" x14ac:dyDescent="0.25">
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>203</v>
       </c>
     </row>
@@ -4118,31 +4120,31 @@
       <c r="B12" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="C12" s="20">
+      <c r="C12" s="21">
         <f t="shared" ref="C12:I12" si="1">SUM(C6:C11)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="21">
         <f t="shared" si="1"/>
         <v>-71</v>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="21">
         <f t="shared" si="1"/>
         <v>-74</v>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="21">
         <f t="shared" si="1"/>
         <v>-7</v>
       </c>
-      <c r="G12" s="20">
+      <c r="G12" s="21">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H12" s="20">
+      <c r="H12" s="21">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I12" s="20">
+      <c r="I12" s="21">
         <f t="shared" si="1"/>
         <v>-152</v>
       </c>
@@ -4178,7 +4180,7 @@
       </c>
     </row>
     <row r="3" spans="2:18" ht="36" x14ac:dyDescent="0.25">
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>214</v>
       </c>
     </row>
@@ -4240,22 +4242,22 @@
         <v>222</v>
       </c>
       <c r="C6" s="15">
-        <v>1143</v>
+        <v>1142.8571428571429</v>
       </c>
       <c r="D6" s="15">
-        <v>795.16</v>
+        <v>794.95478476190488</v>
       </c>
       <c r="E6" s="15">
-        <v>1244.4357</v>
+        <v>1243.9531420571429</v>
       </c>
       <c r="F6" s="15">
-        <v>1298.159676</v>
+        <v>1297.492175906857</v>
       </c>
       <c r="G6" s="15">
-        <v>1353.9870984300001</v>
+        <v>1353.1239939597031</v>
       </c>
       <c r="H6" s="15">
-        <v>1411.9958224974</v>
+        <v>1410.925978137403</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>223</v>
@@ -4285,7 +4287,7 @@
         <v>25</v>
       </c>
       <c r="R6" s="8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.25">
@@ -4296,19 +4298,19 @@
         <v>0</v>
       </c>
       <c r="D7" s="15">
-        <v>54.93333333333333</v>
+        <v>54.362026666666672</v>
       </c>
       <c r="E7" s="15">
-        <v>84.872</v>
+        <v>83.989331199999995</v>
       </c>
       <c r="F7" s="15">
-        <v>87.41816</v>
+        <v>86.509011135999998</v>
       </c>
       <c r="G7" s="15">
-        <v>90.040704800000015</v>
+        <v>89.104281470080011</v>
       </c>
       <c r="H7" s="15">
-        <v>92.741925944000002</v>
+        <v>91.777409914182414</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>230</v>
@@ -4345,27 +4347,27 @@
       <c r="B8" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="23">
         <f>'M3 Stand-alone'!D11</f>
         <v>0</v>
       </c>
-      <c r="D8" s="22">
+      <c r="D8" s="23">
         <f>'M3 Stand-alone'!E11</f>
         <v>-10</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="23">
         <f>'M3 Stand-alone'!F11</f>
         <v>-28</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="23">
         <f>'M3 Stand-alone'!G11</f>
         <v>-40</v>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="23">
         <f>'M3 Stand-alone'!H11</f>
         <v>-40</v>
       </c>
-      <c r="H8" s="22">
+      <c r="H8" s="23">
         <f>'M3 Stand-alone'!I11</f>
         <v>-40</v>
       </c>
@@ -4404,27 +4406,27 @@
       <c r="B9" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="23">
         <f>'M3 Stand-alone'!D12</f>
         <v>0</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="23">
         <f>'M3 Stand-alone'!E12</f>
         <v>-12</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="23">
         <f>'M3 Stand-alone'!F12</f>
         <v>-25.5</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="23">
         <f>'M3 Stand-alone'!G12</f>
         <v>-30</v>
       </c>
-      <c r="G9" s="22">
+      <c r="G9" s="23">
         <f>'M3 Stand-alone'!H12</f>
         <v>-30</v>
       </c>
-      <c r="H9" s="22">
+      <c r="H9" s="23">
         <f>'M3 Stand-alone'!I12</f>
         <v>-30</v>
       </c>
@@ -4463,27 +4465,27 @@
       <c r="B10" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="23">
         <f>'M3 Stand-alone'!D13</f>
         <v>0</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="23">
         <f>'M3 Stand-alone'!E13</f>
         <v>-12.5</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="23">
         <f>'M3 Stand-alone'!F13</f>
         <v>-25</v>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="23">
         <f>'M3 Stand-alone'!G13</f>
         <v>-25</v>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="23">
         <f>'M3 Stand-alone'!H13</f>
         <v>-25</v>
       </c>
-      <c r="H10" s="22">
+      <c r="H10" s="23">
         <f>'M3 Stand-alone'!I13</f>
         <v>-25</v>
       </c>
@@ -4522,27 +4524,27 @@
       <c r="B11" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="23">
         <f>'M3 Stand-alone'!D14</f>
         <v>0</v>
       </c>
-      <c r="D11" s="22">
+      <c r="D11" s="23">
         <f>'M3 Stand-alone'!E14</f>
         <v>-11.25</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="23">
         <f>'M3 Stand-alone'!F14</f>
         <v>-22.5</v>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="23">
         <f>'M3 Stand-alone'!G14</f>
         <v>-25</v>
       </c>
-      <c r="G11" s="22">
+      <c r="G11" s="23">
         <f>'M3 Stand-alone'!H14</f>
         <v>-25</v>
       </c>
-      <c r="H11" s="22">
+      <c r="H11" s="23">
         <f>'M3 Stand-alone'!I14</f>
         <v>-25</v>
       </c>
@@ -4581,27 +4583,27 @@
       <c r="B12" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="23">
         <f>'M4 TSA'!I6</f>
         <v>0</v>
       </c>
-      <c r="D12" s="22">
+      <c r="D12" s="23">
         <f>'M4 TSA'!J6</f>
         <v>-16.8</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="23">
         <f>'M4 TSA'!K6</f>
         <v>-25.20000000000001</v>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="23">
         <f>'M4 TSA'!L6</f>
         <v>-8.4</v>
       </c>
-      <c r="G12" s="22">
+      <c r="G12" s="23">
         <f>'M4 TSA'!M6</f>
         <v>0</v>
       </c>
-      <c r="H12" s="22">
+      <c r="H12" s="23">
         <f>'M4 TSA'!N6</f>
         <v>0</v>
       </c>
@@ -4640,27 +4642,27 @@
       <c r="B13" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="23">
         <f>'M4 TSA'!I7</f>
         <v>0</v>
       </c>
-      <c r="D13" s="22">
+      <c r="D13" s="23">
         <f>'M4 TSA'!J7</f>
         <v>-10</v>
       </c>
-      <c r="E13" s="22">
+      <c r="E13" s="23">
         <f>'M4 TSA'!K7</f>
         <v>-12.5</v>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="23">
         <f>'M4 TSA'!L7</f>
         <v>0</v>
       </c>
-      <c r="G13" s="22">
+      <c r="G13" s="23">
         <f>'M4 TSA'!M7</f>
         <v>0</v>
       </c>
-      <c r="H13" s="22">
+      <c r="H13" s="23">
         <f>'M4 TSA'!N7</f>
         <v>0</v>
       </c>
@@ -4699,27 +4701,27 @@
       <c r="B14" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="23">
         <f>'M4 TSA'!I8</f>
         <v>0</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="23">
         <f>'M4 TSA'!J8</f>
         <v>-6.7999999999999989</v>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="23">
         <f>'M4 TSA'!K8</f>
         <v>-3.4</v>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="23">
         <f>'M4 TSA'!L8</f>
         <v>0</v>
       </c>
-      <c r="G14" s="22">
+      <c r="G14" s="23">
         <f>'M4 TSA'!M8</f>
         <v>0</v>
       </c>
-      <c r="H14" s="22">
+      <c r="H14" s="23">
         <f>'M4 TSA'!N8</f>
         <v>0</v>
       </c>
@@ -4758,27 +4760,27 @@
       <c r="B15" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="C15" s="22">
+      <c r="C15" s="23">
         <f>'M4 TSA'!I9</f>
         <v>0</v>
       </c>
-      <c r="D15" s="22">
+      <c r="D15" s="23">
         <f>'M4 TSA'!J9</f>
         <v>-4</v>
       </c>
-      <c r="E15" s="22">
+      <c r="E15" s="23">
         <f>'M4 TSA'!K9</f>
         <v>-6</v>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="23">
         <f>'M4 TSA'!L9</f>
         <v>-2</v>
       </c>
-      <c r="G15" s="22">
+      <c r="G15" s="23">
         <f>'M4 TSA'!M9</f>
         <v>0</v>
       </c>
-      <c r="H15" s="22">
+      <c r="H15" s="23">
         <f>'M4 TSA'!N9</f>
         <v>0</v>
       </c>
@@ -4817,27 +4819,27 @@
       <c r="B16" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="C16" s="22">
+      <c r="C16" s="23">
         <f>'M4 TSA'!I10</f>
         <v>0</v>
       </c>
-      <c r="D16" s="22">
+      <c r="D16" s="23">
         <f>'M4 TSA'!J10</f>
         <v>-2.4</v>
       </c>
-      <c r="E16" s="22">
+      <c r="E16" s="23">
         <f>'M4 TSA'!K10</f>
         <v>-1.2</v>
       </c>
-      <c r="F16" s="22">
+      <c r="F16" s="23">
         <f>'M4 TSA'!L10</f>
         <v>0</v>
       </c>
-      <c r="G16" s="22">
+      <c r="G16" s="23">
         <f>'M4 TSA'!M10</f>
         <v>0</v>
       </c>
-      <c r="H16" s="22">
+      <c r="H16" s="23">
         <f>'M4 TSA'!N10</f>
         <v>0</v>
       </c>
@@ -4876,27 +4878,27 @@
       <c r="B17" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="C17" s="22">
+      <c r="C17" s="23">
         <f>'M5 One-offs'!C6</f>
         <v>0</v>
       </c>
-      <c r="D17" s="22">
+      <c r="D17" s="23">
         <f>'M5 One-offs'!D6</f>
         <v>-24</v>
       </c>
-      <c r="E17" s="22">
+      <c r="E17" s="23">
         <f>'M5 One-offs'!E6</f>
         <v>-34</v>
       </c>
-      <c r="F17" s="22">
+      <c r="F17" s="23">
         <f>'M5 One-offs'!F6</f>
         <v>0</v>
       </c>
-      <c r="G17" s="22">
+      <c r="G17" s="23">
         <f>'M5 One-offs'!G6</f>
         <v>0</v>
       </c>
-      <c r="H17" s="22">
+      <c r="H17" s="23">
         <f>'M5 One-offs'!H6</f>
         <v>0</v>
       </c>
@@ -4935,27 +4937,27 @@
       <c r="B18" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="C18" s="22">
+      <c r="C18" s="23">
         <f>'M5 One-offs'!C7</f>
         <v>0</v>
       </c>
-      <c r="D18" s="22">
+      <c r="D18" s="23">
         <f>'M5 One-offs'!D7</f>
         <v>-12</v>
       </c>
-      <c r="E18" s="22">
+      <c r="E18" s="23">
         <f>'M5 One-offs'!E7</f>
         <v>-6</v>
       </c>
-      <c r="F18" s="22">
+      <c r="F18" s="23">
         <f>'M5 One-offs'!F7</f>
         <v>0</v>
       </c>
-      <c r="G18" s="22">
+      <c r="G18" s="23">
         <f>'M5 One-offs'!G7</f>
         <v>0</v>
       </c>
-      <c r="H18" s="22">
+      <c r="H18" s="23">
         <f>'M5 One-offs'!H7</f>
         <v>0</v>
       </c>
@@ -4994,27 +4996,27 @@
       <c r="B19" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="C19" s="22">
+      <c r="C19" s="23">
         <f>'M5 One-offs'!C8</f>
         <v>0</v>
       </c>
-      <c r="D19" s="22">
+      <c r="D19" s="23">
         <f>'M5 One-offs'!D8</f>
         <v>-14</v>
       </c>
-      <c r="E19" s="22">
+      <c r="E19" s="23">
         <f>'M5 One-offs'!E8</f>
         <v>-16</v>
       </c>
-      <c r="F19" s="22">
+      <c r="F19" s="23">
         <f>'M5 One-offs'!F8</f>
         <v>-4</v>
       </c>
-      <c r="G19" s="22">
+      <c r="G19" s="23">
         <f>'M5 One-offs'!G8</f>
         <v>0</v>
       </c>
-      <c r="H19" s="22">
+      <c r="H19" s="23">
         <f>'M5 One-offs'!H8</f>
         <v>0</v>
       </c>
@@ -5053,27 +5055,27 @@
       <c r="B20" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="23">
         <f>'M5 One-offs'!C9</f>
         <v>0</v>
       </c>
-      <c r="D20" s="22">
+      <c r="D20" s="23">
         <f>'M5 One-offs'!D9</f>
         <v>-9</v>
       </c>
-      <c r="E20" s="22">
+      <c r="E20" s="23">
         <f>'M5 One-offs'!E9</f>
         <v>-7</v>
       </c>
-      <c r="F20" s="22">
+      <c r="F20" s="23">
         <f>'M5 One-offs'!F9</f>
         <v>0</v>
       </c>
-      <c r="G20" s="22">
+      <c r="G20" s="23">
         <f>'M5 One-offs'!G9</f>
         <v>0</v>
       </c>
-      <c r="H20" s="22">
+      <c r="H20" s="23">
         <f>'M5 One-offs'!H9</f>
         <v>0</v>
       </c>
@@ -5112,27 +5114,27 @@
       <c r="B21" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="23">
         <f>'M5 One-offs'!C10</f>
         <v>0</v>
       </c>
-      <c r="D21" s="22">
+      <c r="D21" s="23">
         <f>'M5 One-offs'!D10</f>
         <v>-4</v>
       </c>
-      <c r="E21" s="22">
+      <c r="E21" s="23">
         <f>'M5 One-offs'!E10</f>
         <v>-7</v>
       </c>
-      <c r="F21" s="22">
+      <c r="F21" s="23">
         <f>'M5 One-offs'!F10</f>
         <v>-3</v>
       </c>
-      <c r="G21" s="22">
+      <c r="G21" s="23">
         <f>'M5 One-offs'!G10</f>
         <v>0</v>
       </c>
-      <c r="H21" s="22">
+      <c r="H21" s="23">
         <f>'M5 One-offs'!H10</f>
         <v>0</v>
       </c>
@@ -5171,27 +5173,27 @@
       <c r="B22" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="C22" s="22">
+      <c r="C22" s="23">
         <f>'M5 One-offs'!C11</f>
         <v>0</v>
       </c>
-      <c r="D22" s="22">
+      <c r="D22" s="23">
         <f>'M5 One-offs'!D11</f>
         <v>-8</v>
       </c>
-      <c r="E22" s="22">
+      <c r="E22" s="23">
         <f>'M5 One-offs'!E11</f>
         <v>-4</v>
       </c>
-      <c r="F22" s="22">
+      <c r="F22" s="23">
         <f>'M5 One-offs'!F11</f>
         <v>0</v>
       </c>
-      <c r="G22" s="22">
+      <c r="G22" s="23">
         <f>'M5 One-offs'!G11</f>
         <v>0</v>
       </c>
-      <c r="H22" s="22">
+      <c r="H22" s="23">
         <f>'M5 One-offs'!H11</f>
         <v>0</v>
       </c>
@@ -5390,22 +5392,22 @@
         <v>265</v>
       </c>
       <c r="C26" s="15">
-        <v>-251.46</v>
+        <v>-251.42857142857139</v>
       </c>
       <c r="D26" s="15">
-        <v>-176.95553333333331</v>
+        <v>-176.78469851428571</v>
       </c>
       <c r="E26" s="15">
-        <v>-270.22769399999999</v>
+        <v>-269.92734411657142</v>
       </c>
       <c r="F26" s="15">
-        <v>-278.42712391999999</v>
+        <v>-278.08026114942862</v>
       </c>
       <c r="G26" s="15">
-        <v>-291.28611671060003</v>
+        <v>-290.89022059455232</v>
       </c>
       <c r="H26" s="15">
-        <v>-304.64230465710801</v>
+        <v>-304.19474537134892</v>
       </c>
       <c r="I26" s="8" t="s">
         <v>257</v>
@@ -5435,7 +5437,7 @@
         <v>25</v>
       </c>
       <c r="R26" s="8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" spans="2:18" x14ac:dyDescent="0.25">
@@ -5488,7 +5490,7 @@
         <v>25</v>
       </c>
       <c r="R27" s="8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="28" spans="2:18" x14ac:dyDescent="0.25">
@@ -5496,22 +5498,22 @@
         <v>269</v>
       </c>
       <c r="C28" s="15">
-        <v>-125</v>
+        <v>-123.7</v>
       </c>
       <c r="D28" s="15">
-        <v>-85.833333333333329</v>
+        <v>-84.940666666666687</v>
       </c>
       <c r="E28" s="15">
-        <v>-132.61250000000001</v>
+        <v>-131.23333</v>
       </c>
       <c r="F28" s="15">
-        <v>-136.59087500000001</v>
+        <v>-135.17032990000001</v>
       </c>
       <c r="G28" s="15">
-        <v>-140.68860125</v>
+        <v>-139.22543979700001</v>
       </c>
       <c r="H28" s="15">
-        <v>-144.90925928749999</v>
+        <v>-143.40220299091001</v>
       </c>
       <c r="I28" s="8" t="s">
         <v>257</v>
@@ -5552,19 +5554,19 @@
         <v>0</v>
       </c>
       <c r="D29" s="15">
-        <v>-15</v>
+        <v>-14.844000000000049</v>
       </c>
       <c r="E29" s="15">
-        <v>-23.175000000000001</v>
+        <v>-22.933979999999931</v>
       </c>
       <c r="F29" s="15">
-        <v>-23.870250000000031</v>
+        <v>-23.6219994</v>
       </c>
       <c r="G29" s="15">
-        <v>-24.58635750000003</v>
+        <v>-24.330659382000071</v>
       </c>
       <c r="H29" s="15">
-        <v>-25.32394822499996</v>
+        <v>-25.06057916346003</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>257</v>
@@ -5654,38 +5656,38 @@
       <c r="B31" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="C31" s="23">
+      <c r="C31" s="24">
         <f t="shared" ref="C31:H31" si="0">SUM(C6:C30)</f>
-        <v>766.54</v>
-      </c>
-      <c r="D31" s="20">
+        <v>767.72857142857151</v>
+      </c>
+      <c r="D31" s="21">
         <f t="shared" si="0"/>
-        <v>364.97446666666679</v>
-      </c>
-      <c r="E31" s="20">
+        <v>365.41744624761924</v>
+      </c>
+      <c r="E31" s="21">
         <f t="shared" si="0"/>
-        <v>676.898506</v>
-      </c>
-      <c r="F31" s="20">
+        <v>677.45381914057123</v>
+      </c>
+      <c r="F31" s="21">
         <f t="shared" si="0"/>
-        <v>823.11758707999979</v>
-      </c>
-      <c r="G31" s="20">
+        <v>823.55659659342814</v>
+      </c>
+      <c r="G31" s="21">
         <f t="shared" si="0"/>
-        <v>917.46672776939988</v>
-      </c>
-      <c r="H31" s="20">
+        <v>917.78195565623059</v>
+      </c>
+      <c r="H31" s="21">
         <f t="shared" si="0"/>
-        <v>909.86223627179209</v>
+        <v>910.04586052586649</v>
       </c>
     </row>
     <row r="33" spans="2:9" ht="123.75" x14ac:dyDescent="0.25">
       <c r="B33" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="C33" s="20">
+      <c r="C33" s="21">
         <f>'M6 Bridge'!H6+'M6 Bridge'!H7+'M3 Stand-alone'!C15</f>
-        <v>1384.7377484414001</v>
+        <v>1382.7033880515855</v>
       </c>
       <c r="I33" s="13" t="s">
         <v>277</v>
@@ -5695,7 +5697,7 @@
       <c r="B34" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="C34" s="20">
+      <c r="C34" s="21">
         <f>-('M4 TSA'!J11+'M5 One-offs'!D12+'M6 Bridge'!D23+'M4 TSA'!K11+'M5 One-offs'!E12+'M6 Bridge'!E23+'M4 TSA'!L11+'M5 One-offs'!F12+'M6 Bridge'!F23+'M4 TSA'!M11+'M5 One-offs'!G12+'M6 Bridge'!G23+'M4 TSA'!N11+'M5 One-offs'!H12+'M6 Bridge'!H23)</f>
         <v>295.7</v>
       </c>
@@ -5729,7 +5731,7 @@
       </c>
     </row>
     <row r="3" spans="2:12" ht="48" x14ac:dyDescent="0.25">
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>281</v>
       </c>
     </row>
@@ -5783,19 +5785,19 @@
         <v>285</v>
       </c>
       <c r="C10" s="15">
-        <v>795.16</v>
+        <v>794.95478476190488</v>
       </c>
       <c r="D10" s="15">
-        <v>1244.4357</v>
+        <v>1243.9531420571429</v>
       </c>
       <c r="E10" s="15">
-        <v>1298.159676</v>
+        <v>1297.492175906857</v>
       </c>
       <c r="F10" s="15">
-        <v>1353.9870984300001</v>
+        <v>1353.1239939597031</v>
       </c>
       <c r="G10" s="15">
-        <v>1411.9958224974</v>
+        <v>1410.925978137403</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>226</v>
@@ -5807,7 +5809,7 @@
         <v>25</v>
       </c>
       <c r="K10" s="8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="L10" s="13" t="s">
         <v>286</v>
@@ -5818,19 +5820,19 @@
         <v>287</v>
       </c>
       <c r="C11" s="15">
-        <v>-174.93520000000001</v>
+        <v>-174.89005264761909</v>
       </c>
       <c r="D11" s="15">
-        <v>-273.77585399999998</v>
+        <v>-273.66969125257151</v>
       </c>
       <c r="E11" s="15">
-        <v>-285.59512871999999</v>
+        <v>-285.44827869950859</v>
       </c>
       <c r="F11" s="15">
-        <v>-297.8771616546</v>
+        <v>-297.68727867113472</v>
       </c>
       <c r="G11" s="15">
-        <v>-310.63908094942798</v>
+        <v>-310.40371519022881</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>226</v>
@@ -5842,7 +5844,7 @@
         <v>25</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="L11" s="13" t="s">
         <v>288</v>
@@ -5853,19 +5855,19 @@
         <v>289</v>
       </c>
       <c r="C12" s="15">
-        <v>-85.833333333333329</v>
+        <v>-84.940666666666687</v>
       </c>
       <c r="D12" s="15">
-        <v>-132.61250000000001</v>
+        <v>-131.23333</v>
       </c>
       <c r="E12" s="15">
-        <v>-136.59087500000001</v>
+        <v>-135.17032990000001</v>
       </c>
       <c r="F12" s="15">
-        <v>-140.68860125</v>
+        <v>-139.22543979700001</v>
       </c>
       <c r="G12" s="15">
-        <v>-144.90925928749999</v>
+        <v>-143.40220299091001</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>226</v>
@@ -5888,19 +5890,19 @@
         <v>291</v>
       </c>
       <c r="C13" s="15">
-        <v>-15</v>
+        <v>-14.844000000000049</v>
       </c>
       <c r="D13" s="15">
-        <v>-23.175000000000001</v>
+        <v>-22.933979999999931</v>
       </c>
       <c r="E13" s="15">
-        <v>-23.870250000000031</v>
+        <v>-23.6219994</v>
       </c>
       <c r="F13" s="15">
-        <v>-24.58635750000003</v>
+        <v>-24.330659382000071</v>
       </c>
       <c r="G13" s="15">
-        <v>-25.32394822499996</v>
+        <v>-25.06057916346003</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>226</v>
@@ -5957,25 +5959,25 @@
       <c r="B15" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="C15" s="20">
+      <c r="C15" s="21">
         <f>SUM(C10:C14)</f>
-        <v>519.39146666666659</v>
-      </c>
-      <c r="D15" s="20">
+        <v>520.28006544761911</v>
+      </c>
+      <c r="D15" s="21">
         <f>SUM(D10:D14)</f>
-        <v>814.87234600000011</v>
-      </c>
-      <c r="E15" s="20">
+        <v>816.1161408045715</v>
+      </c>
+      <c r="E15" s="21">
         <f>SUM(E10:E14)</f>
-        <v>852.1034222799999</v>
-      </c>
-      <c r="F15" s="20">
+        <v>853.25156790734832</v>
+      </c>
+      <c r="F15" s="21">
         <f>SUM(F10:F14)</f>
-        <v>890.83497802539989</v>
-      </c>
-      <c r="G15" s="20">
+        <v>891.88061610956834</v>
+      </c>
+      <c r="G15" s="21">
         <f>SUM(G10:G14)</f>
-        <v>931.12353403547206</v>
+        <v>932.05948079280404</v>
       </c>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
@@ -6024,7 +6026,7 @@
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="25" t="s">
         <v>299</v>
       </c>
     </row>
@@ -6032,25 +6034,25 @@
       <c r="B23" s="6" t="s">
         <v>300</v>
       </c>
-      <c r="C23" s="22">
+      <c r="C23" s="23">
         <f>-'M6 Bridge'!D6</f>
-        <v>-795.16</v>
-      </c>
-      <c r="D23" s="22">
+        <v>-794.95478476190488</v>
+      </c>
+      <c r="D23" s="23">
         <f>-'M6 Bridge'!E6</f>
-        <v>-1244.4357</v>
-      </c>
-      <c r="E23" s="22">
+        <v>-1243.9531420571429</v>
+      </c>
+      <c r="E23" s="23">
         <f>-'M6 Bridge'!F6</f>
-        <v>-1298.159676</v>
-      </c>
-      <c r="F23" s="22">
+        <v>-1297.492175906857</v>
+      </c>
+      <c r="F23" s="23">
         <f>-'M6 Bridge'!G6</f>
-        <v>-1353.9870984300001</v>
-      </c>
-      <c r="G23" s="22">
+        <v>-1353.1239939597031</v>
+      </c>
+      <c r="G23" s="23">
         <f>-'M6 Bridge'!H6</f>
-        <v>-1411.9958224974</v>
+        <v>-1410.925978137403</v>
       </c>
       <c r="H23" s="8" t="s">
         <v>226</v>
@@ -6072,25 +6074,25 @@
       <c r="B24" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="C24" s="22">
+      <c r="C24" s="23">
         <f>-'M6 Bridge'!D7</f>
-        <v>-54.93333333333333</v>
-      </c>
-      <c r="D24" s="22">
+        <v>-54.362026666666672</v>
+      </c>
+      <c r="D24" s="23">
         <f>-'M6 Bridge'!E7</f>
-        <v>-84.872</v>
-      </c>
-      <c r="E24" s="22">
+        <v>-83.989331199999995</v>
+      </c>
+      <c r="E24" s="23">
         <f>-'M6 Bridge'!F7</f>
-        <v>-87.41816</v>
-      </c>
-      <c r="F24" s="22">
+        <v>-86.509011135999998</v>
+      </c>
+      <c r="F24" s="23">
         <f>-'M6 Bridge'!G7</f>
-        <v>-90.040704800000015</v>
-      </c>
-      <c r="G24" s="22">
+        <v>-89.104281470080011</v>
+      </c>
+      <c r="G24" s="23">
         <f>-'M6 Bridge'!H7</f>
-        <v>-92.741925944000002</v>
+        <v>-91.777409914182414</v>
       </c>
       <c r="H24" s="8" t="s">
         <v>226</v>
@@ -6112,23 +6114,23 @@
       <c r="B25" s="6" t="s">
         <v>302</v>
       </c>
-      <c r="C25" s="22">
+      <c r="C25" s="23">
         <f>-'M6 Bridge'!D8</f>
         <v>10</v>
       </c>
-      <c r="D25" s="22">
+      <c r="D25" s="23">
         <f>-'M6 Bridge'!E8</f>
         <v>28</v>
       </c>
-      <c r="E25" s="22">
+      <c r="E25" s="23">
         <f>-'M6 Bridge'!F8</f>
         <v>40</v>
       </c>
-      <c r="F25" s="22">
+      <c r="F25" s="23">
         <f>-'M6 Bridge'!G8</f>
         <v>40</v>
       </c>
-      <c r="G25" s="22">
+      <c r="G25" s="23">
         <f>-'M6 Bridge'!H8</f>
         <v>40</v>
       </c>
@@ -6152,23 +6154,23 @@
       <c r="B26" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="C26" s="22">
+      <c r="C26" s="23">
         <f>-'M6 Bridge'!D9</f>
         <v>12</v>
       </c>
-      <c r="D26" s="22">
+      <c r="D26" s="23">
         <f>-'M6 Bridge'!E9</f>
         <v>25.5</v>
       </c>
-      <c r="E26" s="22">
+      <c r="E26" s="23">
         <f>-'M6 Bridge'!F9</f>
         <v>30</v>
       </c>
-      <c r="F26" s="22">
+      <c r="F26" s="23">
         <f>-'M6 Bridge'!G9</f>
         <v>30</v>
       </c>
-      <c r="G26" s="22">
+      <c r="G26" s="23">
         <f>-'M6 Bridge'!H9</f>
         <v>30</v>
       </c>
@@ -6192,23 +6194,23 @@
       <c r="B27" s="6" t="s">
         <v>304</v>
       </c>
-      <c r="C27" s="22">
+      <c r="C27" s="23">
         <f>-'M6 Bridge'!D10</f>
         <v>12.5</v>
       </c>
-      <c r="D27" s="22">
+      <c r="D27" s="23">
         <f>-'M6 Bridge'!E10</f>
         <v>25</v>
       </c>
-      <c r="E27" s="22">
+      <c r="E27" s="23">
         <f>-'M6 Bridge'!F10</f>
         <v>25</v>
       </c>
-      <c r="F27" s="22">
+      <c r="F27" s="23">
         <f>-'M6 Bridge'!G10</f>
         <v>25</v>
       </c>
-      <c r="G27" s="22">
+      <c r="G27" s="23">
         <f>-'M6 Bridge'!H10</f>
         <v>25</v>
       </c>
@@ -6232,23 +6234,23 @@
       <c r="B28" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="C28" s="22">
+      <c r="C28" s="23">
         <f>-'M6 Bridge'!D11</f>
         <v>11.25</v>
       </c>
-      <c r="D28" s="22">
+      <c r="D28" s="23">
         <f>-'M6 Bridge'!E11</f>
         <v>22.5</v>
       </c>
-      <c r="E28" s="22">
+      <c r="E28" s="23">
         <f>-'M6 Bridge'!F11</f>
         <v>25</v>
       </c>
-      <c r="F28" s="22">
+      <c r="F28" s="23">
         <f>-'M6 Bridge'!G11</f>
         <v>25</v>
       </c>
-      <c r="G28" s="22">
+      <c r="G28" s="23">
         <f>-'M6 Bridge'!H11</f>
         <v>25</v>
       </c>
@@ -6272,25 +6274,25 @@
       <c r="B29" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="C29" s="22">
+      <c r="C29" s="23">
         <f>-'M6 Bridge'!D26</f>
-        <v>176.95553333333331</v>
-      </c>
-      <c r="D29" s="22">
+        <v>176.78469851428571</v>
+      </c>
+      <c r="D29" s="23">
         <f>-'M6 Bridge'!E26</f>
-        <v>270.22769399999999</v>
-      </c>
-      <c r="E29" s="22">
+        <v>269.92734411657142</v>
+      </c>
+      <c r="E29" s="23">
         <f>-'M6 Bridge'!F26</f>
-        <v>278.42712391999999</v>
-      </c>
-      <c r="F29" s="22">
+        <v>278.08026114942862</v>
+      </c>
+      <c r="F29" s="23">
         <f>-'M6 Bridge'!G26</f>
-        <v>291.28611671060003</v>
-      </c>
-      <c r="G29" s="22">
+        <v>290.89022059455232</v>
+      </c>
+      <c r="G29" s="23">
         <f>-'M6 Bridge'!H26</f>
-        <v>304.64230465710801</v>
+        <v>304.19474537134892</v>
       </c>
       <c r="H29" s="8" t="s">
         <v>226</v>
@@ -6312,25 +6314,25 @@
       <c r="B30" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="C30" s="22">
+      <c r="C30" s="23">
         <f>-'M6 Bridge'!D28</f>
-        <v>85.833333333333329</v>
-      </c>
-      <c r="D30" s="22">
+        <v>84.940666666666687</v>
+      </c>
+      <c r="D30" s="23">
         <f>-'M6 Bridge'!E28</f>
-        <v>132.61250000000001</v>
-      </c>
-      <c r="E30" s="22">
+        <v>131.23333</v>
+      </c>
+      <c r="E30" s="23">
         <f>-'M6 Bridge'!F28</f>
-        <v>136.59087500000001</v>
-      </c>
-      <c r="F30" s="22">
+        <v>135.17032990000001</v>
+      </c>
+      <c r="F30" s="23">
         <f>-'M6 Bridge'!G28</f>
-        <v>140.68860125</v>
-      </c>
-      <c r="G30" s="22">
+        <v>139.22543979700001</v>
+      </c>
+      <c r="G30" s="23">
         <f>-'M6 Bridge'!H28</f>
-        <v>144.90925928749999</v>
+        <v>143.40220299091001</v>
       </c>
       <c r="H30" s="8" t="s">
         <v>226</v>
@@ -6352,25 +6354,25 @@
       <c r="B31" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="C31" s="22">
+      <c r="C31" s="23">
         <f>-'M6 Bridge'!D29</f>
-        <v>15</v>
-      </c>
-      <c r="D31" s="22">
+        <v>14.844000000000049</v>
+      </c>
+      <c r="D31" s="23">
         <f>-'M6 Bridge'!E29</f>
-        <v>23.175000000000001</v>
-      </c>
-      <c r="E31" s="22">
+        <v>22.933979999999931</v>
+      </c>
+      <c r="E31" s="23">
         <f>-'M6 Bridge'!F29</f>
-        <v>23.870250000000031</v>
-      </c>
-      <c r="F31" s="22">
+        <v>23.6219994</v>
+      </c>
+      <c r="F31" s="23">
         <f>-'M6 Bridge'!G29</f>
-        <v>24.58635750000003</v>
-      </c>
-      <c r="G31" s="22">
+        <v>24.330659382000071</v>
+      </c>
+      <c r="G31" s="23">
         <f>-'M6 Bridge'!H29</f>
-        <v>25.32394822499996</v>
+        <v>25.06057916346003</v>
       </c>
       <c r="H31" s="8" t="s">
         <v>226</v>
@@ -6392,23 +6394,23 @@
       <c r="B32" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="C32" s="22">
+      <c r="C32" s="23">
         <f>-'M6 Bridge'!D30</f>
         <v>0</v>
       </c>
-      <c r="D32" s="22">
+      <c r="D32" s="23">
         <f>-'M6 Bridge'!E30</f>
         <v>0</v>
       </c>
-      <c r="E32" s="22">
+      <c r="E32" s="23">
         <f>-'M6 Bridge'!F30</f>
         <v>0</v>
       </c>
-      <c r="F32" s="22">
+      <c r="F32" s="23">
         <f>-'M6 Bridge'!G30</f>
         <v>0</v>
       </c>
-      <c r="G32" s="22">
+      <c r="G32" s="23">
         <f>-'M6 Bridge'!H30</f>
         <v>0</v>
       </c>
@@ -6432,25 +6434,25 @@
       <c r="B33" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="C33" s="22">
+      <c r="C33" s="23">
         <f>+'M7 Financement'!C10</f>
-        <v>795.16</v>
-      </c>
-      <c r="D33" s="22">
+        <v>794.95478476190488</v>
+      </c>
+      <c r="D33" s="23">
         <f>+'M7 Financement'!D10</f>
-        <v>1244.4357</v>
-      </c>
-      <c r="E33" s="22">
+        <v>1243.9531420571429</v>
+      </c>
+      <c r="E33" s="23">
         <f>+'M7 Financement'!E10</f>
-        <v>1298.159676</v>
-      </c>
-      <c r="F33" s="22">
+        <v>1297.492175906857</v>
+      </c>
+      <c r="F33" s="23">
         <f>+'M7 Financement'!F10</f>
-        <v>1353.9870984300001</v>
-      </c>
-      <c r="G33" s="22">
+        <v>1353.1239939597031</v>
+      </c>
+      <c r="G33" s="23">
         <f>+'M7 Financement'!G10</f>
-        <v>1411.9958224974</v>
+        <v>1410.925978137403</v>
       </c>
       <c r="H33" s="8" t="s">
         <v>226</v>
@@ -6472,25 +6474,25 @@
       <c r="B34" s="6" t="s">
         <v>313</v>
       </c>
-      <c r="C34" s="22">
+      <c r="C34" s="23">
         <f>+'M7 Financement'!C11</f>
-        <v>-174.93520000000001</v>
-      </c>
-      <c r="D34" s="22">
+        <v>-174.89005264761909</v>
+      </c>
+      <c r="D34" s="23">
         <f>+'M7 Financement'!D11</f>
-        <v>-273.77585399999998</v>
-      </c>
-      <c r="E34" s="22">
+        <v>-273.66969125257151</v>
+      </c>
+      <c r="E34" s="23">
         <f>+'M7 Financement'!E11</f>
-        <v>-285.59512871999999</v>
-      </c>
-      <c r="F34" s="22">
+        <v>-285.44827869950859</v>
+      </c>
+      <c r="F34" s="23">
         <f>+'M7 Financement'!F11</f>
-        <v>-297.8771616546</v>
-      </c>
-      <c r="G34" s="22">
+        <v>-297.68727867113472</v>
+      </c>
+      <c r="G34" s="23">
         <f>+'M7 Financement'!G11</f>
-        <v>-310.63908094942798</v>
+        <v>-310.40371519022881</v>
       </c>
       <c r="H34" s="8" t="s">
         <v>226</v>
@@ -6512,25 +6514,25 @@
       <c r="B35" s="6" t="s">
         <v>314</v>
       </c>
-      <c r="C35" s="22">
+      <c r="C35" s="23">
         <f>+'M7 Financement'!C12</f>
-        <v>-85.833333333333329</v>
-      </c>
-      <c r="D35" s="22">
+        <v>-84.940666666666687</v>
+      </c>
+      <c r="D35" s="23">
         <f>+'M7 Financement'!D12</f>
-        <v>-132.61250000000001</v>
-      </c>
-      <c r="E35" s="22">
+        <v>-131.23333</v>
+      </c>
+      <c r="E35" s="23">
         <f>+'M7 Financement'!E12</f>
-        <v>-136.59087500000001</v>
-      </c>
-      <c r="F35" s="22">
+        <v>-135.17032990000001</v>
+      </c>
+      <c r="F35" s="23">
         <f>+'M7 Financement'!F12</f>
-        <v>-140.68860125</v>
-      </c>
-      <c r="G35" s="22">
+        <v>-139.22543979700001</v>
+      </c>
+      <c r="G35" s="23">
         <f>+'M7 Financement'!G12</f>
-        <v>-144.90925928749999</v>
+        <v>-143.40220299091001</v>
       </c>
       <c r="H35" s="8" t="s">
         <v>226</v>
@@ -6552,25 +6554,25 @@
       <c r="B36" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="C36" s="22">
+      <c r="C36" s="23">
         <f>+'M7 Financement'!C13</f>
-        <v>-15</v>
-      </c>
-      <c r="D36" s="22">
+        <v>-14.844000000000049</v>
+      </c>
+      <c r="D36" s="23">
         <f>+'M7 Financement'!D13</f>
-        <v>-23.175000000000001</v>
-      </c>
-      <c r="E36" s="22">
+        <v>-22.933979999999931</v>
+      </c>
+      <c r="E36" s="23">
         <f>+'M7 Financement'!E13</f>
-        <v>-23.870250000000031</v>
-      </c>
-      <c r="F36" s="22">
+        <v>-23.6219994</v>
+      </c>
+      <c r="F36" s="23">
         <f>+'M7 Financement'!F13</f>
-        <v>-24.58635750000003</v>
-      </c>
-      <c r="G36" s="22">
+        <v>-24.330659382000071</v>
+      </c>
+      <c r="G36" s="23">
         <f>+'M7 Financement'!G13</f>
-        <v>-25.32394822499996</v>
+        <v>-25.06057916346003</v>
       </c>
       <c r="H36" s="8" t="s">
         <v>226</v>
@@ -6592,23 +6594,23 @@
       <c r="B37" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="C37" s="22">
+      <c r="C37" s="23">
         <f>+'M7 Financement'!C14</f>
         <v>0</v>
       </c>
-      <c r="D37" s="22">
+      <c r="D37" s="23">
         <f>+'M7 Financement'!D14</f>
         <v>0</v>
       </c>
-      <c r="E37" s="22">
+      <c r="E37" s="23">
         <f>+'M7 Financement'!E14</f>
         <v>0</v>
       </c>
-      <c r="F37" s="22">
+      <c r="F37" s="23">
         <f>+'M7 Financement'!F14</f>
         <v>0</v>
       </c>
-      <c r="G37" s="22">
+      <c r="G37" s="23">
         <f>+'M7 Financement'!G14</f>
         <v>0</v>
       </c>
@@ -6632,29 +6634,29 @@
       <c r="B38" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="C38" s="20">
+      <c r="C38" s="21">
         <f>SUM(C23:C37)</f>
-        <v>-7.1629999999999683</v>
-      </c>
-      <c r="D38" s="20">
+        <v>-6.7173808000000559</v>
+      </c>
+      <c r="D38" s="21">
         <f>SUM(D23:D37)</f>
-        <v>12.579839999999773</v>
-      </c>
-      <c r="E38" s="20">
+        <v>13.268321664000045</v>
+      </c>
+      <c r="E38" s="21">
         <f>SUM(E23:E37)</f>
-        <v>25.413835200000047</v>
-      </c>
-      <c r="F38" s="20">
+        <v>26.122971313920168</v>
+      </c>
+      <c r="F38" s="21">
         <f>SUM(F23:F37)</f>
-        <v>23.368250256000142</v>
-      </c>
-      <c r="G38" s="20">
+        <v>24.098660453337665</v>
+      </c>
+      <c r="G38" s="21">
         <f>SUM(G23:G37)</f>
-        <v>21.261297763679998</v>
+        <v>22.013620266937696</v>
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B40" s="24" t="s">
+      <c r="B40" s="25" t="s">
         <v>318</v>
       </c>
     </row>
@@ -6662,23 +6664,23 @@
       <c r="B41" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="C41" s="22">
+      <c r="C41" s="23">
         <f>-'M6 Bridge'!D12</f>
         <v>16.8</v>
       </c>
-      <c r="D41" s="22">
+      <c r="D41" s="23">
         <f>-'M6 Bridge'!E12</f>
         <v>25.20000000000001</v>
       </c>
-      <c r="E41" s="22">
+      <c r="E41" s="23">
         <f>-'M6 Bridge'!F12</f>
         <v>8.4</v>
       </c>
-      <c r="F41" s="22">
+      <c r="F41" s="23">
         <f>-'M6 Bridge'!G12</f>
         <v>0</v>
       </c>
-      <c r="G41" s="22">
+      <c r="G41" s="23">
         <f>-'M6 Bridge'!H12</f>
         <v>0</v>
       </c>
@@ -6702,23 +6704,23 @@
       <c r="B42" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="C42" s="22">
+      <c r="C42" s="23">
         <f>-'M6 Bridge'!D13</f>
         <v>10</v>
       </c>
-      <c r="D42" s="22">
+      <c r="D42" s="23">
         <f>-'M6 Bridge'!E13</f>
         <v>12.5</v>
       </c>
-      <c r="E42" s="22">
+      <c r="E42" s="23">
         <f>-'M6 Bridge'!F13</f>
         <v>0</v>
       </c>
-      <c r="F42" s="22">
+      <c r="F42" s="23">
         <f>-'M6 Bridge'!G13</f>
         <v>0</v>
       </c>
-      <c r="G42" s="22">
+      <c r="G42" s="23">
         <f>-'M6 Bridge'!H13</f>
         <v>0</v>
       </c>
@@ -6742,23 +6744,23 @@
       <c r="B43" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="C43" s="22">
+      <c r="C43" s="23">
         <f>-'M6 Bridge'!D14</f>
         <v>6.7999999999999989</v>
       </c>
-      <c r="D43" s="22">
+      <c r="D43" s="23">
         <f>-'M6 Bridge'!E14</f>
         <v>3.4</v>
       </c>
-      <c r="E43" s="22">
+      <c r="E43" s="23">
         <f>-'M6 Bridge'!F14</f>
         <v>0</v>
       </c>
-      <c r="F43" s="22">
+      <c r="F43" s="23">
         <f>-'M6 Bridge'!G14</f>
         <v>0</v>
       </c>
-      <c r="G43" s="22">
+      <c r="G43" s="23">
         <f>-'M6 Bridge'!H14</f>
         <v>0</v>
       </c>
@@ -6782,23 +6784,23 @@
       <c r="B44" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="C44" s="22">
+      <c r="C44" s="23">
         <f>-'M6 Bridge'!D15</f>
         <v>4</v>
       </c>
-      <c r="D44" s="22">
+      <c r="D44" s="23">
         <f>-'M6 Bridge'!E15</f>
         <v>6</v>
       </c>
-      <c r="E44" s="22">
+      <c r="E44" s="23">
         <f>-'M6 Bridge'!F15</f>
         <v>2</v>
       </c>
-      <c r="F44" s="22">
+      <c r="F44" s="23">
         <f>-'M6 Bridge'!G15</f>
         <v>0</v>
       </c>
-      <c r="G44" s="22">
+      <c r="G44" s="23">
         <f>-'M6 Bridge'!H15</f>
         <v>0</v>
       </c>
@@ -6822,23 +6824,23 @@
       <c r="B45" s="6" t="s">
         <v>323</v>
       </c>
-      <c r="C45" s="22">
+      <c r="C45" s="23">
         <f>-'M6 Bridge'!D16</f>
         <v>2.4</v>
       </c>
-      <c r="D45" s="22">
+      <c r="D45" s="23">
         <f>-'M6 Bridge'!E16</f>
         <v>1.2</v>
       </c>
-      <c r="E45" s="22">
+      <c r="E45" s="23">
         <f>-'M6 Bridge'!F16</f>
         <v>0</v>
       </c>
-      <c r="F45" s="22">
+      <c r="F45" s="23">
         <f>-'M6 Bridge'!G16</f>
         <v>0</v>
       </c>
-      <c r="G45" s="22">
+      <c r="G45" s="23">
         <f>-'M6 Bridge'!H16</f>
         <v>0</v>
       </c>
@@ -6862,23 +6864,23 @@
       <c r="B46" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="C46" s="22">
+      <c r="C46" s="23">
         <f>-'M6 Bridge'!D17</f>
         <v>24</v>
       </c>
-      <c r="D46" s="22">
+      <c r="D46" s="23">
         <f>-'M6 Bridge'!E17</f>
         <v>34</v>
       </c>
-      <c r="E46" s="22">
+      <c r="E46" s="23">
         <f>-'M6 Bridge'!F17</f>
         <v>0</v>
       </c>
-      <c r="F46" s="22">
+      <c r="F46" s="23">
         <f>-'M6 Bridge'!G17</f>
         <v>0</v>
       </c>
-      <c r="G46" s="22">
+      <c r="G46" s="23">
         <f>-'M6 Bridge'!H17</f>
         <v>0</v>
       </c>
@@ -6902,23 +6904,23 @@
       <c r="B47" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="C47" s="22">
+      <c r="C47" s="23">
         <f>-'M6 Bridge'!D18</f>
         <v>12</v>
       </c>
-      <c r="D47" s="22">
+      <c r="D47" s="23">
         <f>-'M6 Bridge'!E18</f>
         <v>6</v>
       </c>
-      <c r="E47" s="22">
+      <c r="E47" s="23">
         <f>-'M6 Bridge'!F18</f>
         <v>0</v>
       </c>
-      <c r="F47" s="22">
+      <c r="F47" s="23">
         <f>-'M6 Bridge'!G18</f>
         <v>0</v>
       </c>
-      <c r="G47" s="22">
+      <c r="G47" s="23">
         <f>-'M6 Bridge'!H18</f>
         <v>0</v>
       </c>
@@ -6942,23 +6944,23 @@
       <c r="B48" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="C48" s="22">
+      <c r="C48" s="23">
         <f>-'M6 Bridge'!D19</f>
         <v>14</v>
       </c>
-      <c r="D48" s="22">
+      <c r="D48" s="23">
         <f>-'M6 Bridge'!E19</f>
         <v>16</v>
       </c>
-      <c r="E48" s="22">
+      <c r="E48" s="23">
         <f>-'M6 Bridge'!F19</f>
         <v>4</v>
       </c>
-      <c r="F48" s="22">
+      <c r="F48" s="23">
         <f>-'M6 Bridge'!G19</f>
         <v>0</v>
       </c>
-      <c r="G48" s="22">
+      <c r="G48" s="23">
         <f>-'M6 Bridge'!H19</f>
         <v>0</v>
       </c>
@@ -6982,23 +6984,23 @@
       <c r="B49" s="6" t="s">
         <v>327</v>
       </c>
-      <c r="C49" s="22">
+      <c r="C49" s="23">
         <f>-'M6 Bridge'!D20</f>
         <v>9</v>
       </c>
-      <c r="D49" s="22">
+      <c r="D49" s="23">
         <f>-'M6 Bridge'!E20</f>
         <v>7</v>
       </c>
-      <c r="E49" s="22">
+      <c r="E49" s="23">
         <f>-'M6 Bridge'!F20</f>
         <v>0</v>
       </c>
-      <c r="F49" s="22">
+      <c r="F49" s="23">
         <f>-'M6 Bridge'!G20</f>
         <v>0</v>
       </c>
-      <c r="G49" s="22">
+      <c r="G49" s="23">
         <f>-'M6 Bridge'!H20</f>
         <v>0</v>
       </c>
@@ -7022,23 +7024,23 @@
       <c r="B50" s="6" t="s">
         <v>328</v>
       </c>
-      <c r="C50" s="22">
+      <c r="C50" s="23">
         <f>-'M6 Bridge'!D21</f>
         <v>4</v>
       </c>
-      <c r="D50" s="22">
+      <c r="D50" s="23">
         <f>-'M6 Bridge'!E21</f>
         <v>7</v>
       </c>
-      <c r="E50" s="22">
+      <c r="E50" s="23">
         <f>-'M6 Bridge'!F21</f>
         <v>3</v>
       </c>
-      <c r="F50" s="22">
+      <c r="F50" s="23">
         <f>-'M6 Bridge'!G21</f>
         <v>0</v>
       </c>
-      <c r="G50" s="22">
+      <c r="G50" s="23">
         <f>-'M6 Bridge'!H21</f>
         <v>0</v>
       </c>
@@ -7062,23 +7064,23 @@
       <c r="B51" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="C51" s="22">
+      <c r="C51" s="23">
         <f>-'M6 Bridge'!D22</f>
         <v>8</v>
       </c>
-      <c r="D51" s="22">
+      <c r="D51" s="23">
         <f>-'M6 Bridge'!E22</f>
         <v>4</v>
       </c>
-      <c r="E51" s="22">
+      <c r="E51" s="23">
         <f>-'M6 Bridge'!F22</f>
         <v>0</v>
       </c>
-      <c r="F51" s="22">
+      <c r="F51" s="23">
         <f>-'M6 Bridge'!G22</f>
         <v>0</v>
       </c>
-      <c r="G51" s="22">
+      <c r="G51" s="23">
         <f>-'M6 Bridge'!H22</f>
         <v>0</v>
       </c>
@@ -7102,23 +7104,23 @@
       <c r="B52" s="6" t="s">
         <v>330</v>
       </c>
-      <c r="C52" s="22">
+      <c r="C52" s="23">
         <f>-'M6 Bridge'!D23</f>
         <v>20</v>
       </c>
-      <c r="D52" s="22">
+      <c r="D52" s="23">
         <f>-'M6 Bridge'!E23</f>
         <v>20</v>
       </c>
-      <c r="E52" s="22">
+      <c r="E52" s="23">
         <f>-'M6 Bridge'!F23</f>
         <v>5</v>
       </c>
-      <c r="F52" s="22">
+      <c r="F52" s="23">
         <f>-'M6 Bridge'!G23</f>
         <v>0</v>
       </c>
-      <c r="G52" s="22">
+      <c r="G52" s="23">
         <f>-'M6 Bridge'!H23</f>
         <v>0</v>
       </c>
@@ -7142,23 +7144,23 @@
       <c r="B53" s="6" t="s">
         <v>331</v>
       </c>
-      <c r="C53" s="22">
+      <c r="C53" s="23">
         <f>-'M6 Bridge'!D24</f>
         <v>55</v>
       </c>
-      <c r="D53" s="22">
+      <c r="D53" s="23">
         <f>-'M6 Bridge'!E24</f>
         <v>10</v>
       </c>
-      <c r="E53" s="22">
+      <c r="E53" s="23">
         <f>-'M6 Bridge'!F24</f>
         <v>0</v>
       </c>
-      <c r="F53" s="22">
+      <c r="F53" s="23">
         <f>-'M6 Bridge'!G24</f>
         <v>0</v>
       </c>
-      <c r="G53" s="22">
+      <c r="G53" s="23">
         <f>-'M6 Bridge'!H24</f>
         <v>0</v>
       </c>
@@ -7182,23 +7184,23 @@
       <c r="B54" s="6" t="s">
         <v>332</v>
       </c>
-      <c r="C54" s="22">
+      <c r="C54" s="23">
         <f>-'M6 Bridge'!D25</f>
         <v>0</v>
       </c>
-      <c r="D54" s="22">
+      <c r="D54" s="23">
         <f>-'M6 Bridge'!E25</f>
         <v>0</v>
       </c>
-      <c r="E54" s="22">
+      <c r="E54" s="23">
         <f>-'M6 Bridge'!F25</f>
         <v>-15</v>
       </c>
-      <c r="F54" s="22">
+      <c r="F54" s="23">
         <f>-'M6 Bridge'!G25</f>
         <v>-50</v>
       </c>
-      <c r="G54" s="22">
+      <c r="G54" s="23">
         <f>-'M6 Bridge'!H25</f>
         <v>0</v>
       </c>
@@ -7222,23 +7224,23 @@
       <c r="B55" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="C55" s="22">
+      <c r="C55" s="23">
         <f>-'M6 Bridge'!D27</f>
         <v>-24.42</v>
       </c>
-      <c r="D55" s="22">
+      <c r="D55" s="23">
         <f>-'M6 Bridge'!E27</f>
         <v>-26.905999999999999</v>
       </c>
-      <c r="E55" s="22">
+      <c r="E55" s="23">
         <f>-'M6 Bridge'!F27</f>
         <v>-3.8279999999999998</v>
       </c>
-      <c r="F55" s="22">
+      <c r="F55" s="23">
         <f>-'M6 Bridge'!G27</f>
         <v>0</v>
       </c>
-      <c r="G55" s="22">
+      <c r="G55" s="23">
         <f>-'M6 Bridge'!H27</f>
         <v>0</v>
       </c>
@@ -7262,23 +7264,23 @@
       <c r="B56" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="C56" s="20">
+      <c r="C56" s="21">
         <f>SUM(C41:C55)</f>
         <v>161.57999999999998</v>
       </c>
-      <c r="D56" s="20">
+      <c r="D56" s="21">
         <f>SUM(D41:D55)</f>
         <v>125.39400000000001</v>
       </c>
-      <c r="E56" s="20">
+      <c r="E56" s="21">
         <f>SUM(E41:E55)</f>
         <v>3.5719999999999987</v>
       </c>
-      <c r="F56" s="20">
+      <c r="F56" s="21">
         <f>SUM(F41:F55)</f>
         <v>-50</v>
       </c>
-      <c r="G56" s="20">
+      <c r="G56" s="21">
         <f>SUM(G41:G55)</f>
         <v>0</v>
       </c>
@@ -7314,23 +7316,23 @@
       </c>
       <c r="C61" s="15">
         <f>'M6 Bridge'!D31-'M7 Financement'!C15</f>
-        <v>-154.4169999999998</v>
+        <v>-154.86261919999987</v>
       </c>
       <c r="D61" s="15">
         <f>'M6 Bridge'!E31-'M7 Financement'!D15</f>
-        <v>-137.97384000000011</v>
+        <v>-138.66232166400027</v>
       </c>
       <c r="E61" s="15">
         <f>'M6 Bridge'!F31-'M7 Financement'!E15</f>
-        <v>-28.98583520000011</v>
+        <v>-29.694971313920178</v>
       </c>
       <c r="F61" s="15">
         <f>'M6 Bridge'!G31-'M7 Financement'!F15</f>
-        <v>26.63174974399999</v>
+        <v>25.901339546662257</v>
       </c>
       <c r="G61" s="15">
         <f>'M6 Bridge'!H31-'M7 Financement'!G15</f>
-        <v>-21.261297763679977</v>
+        <v>-22.013620266937551</v>
       </c>
     </row>
     <row r="62" spans="2:12" x14ac:dyDescent="0.25">
@@ -7339,121 +7341,121 @@
       </c>
       <c r="C62" s="15">
         <f>-'M7 Financement'!C61</f>
-        <v>154.4169999999998</v>
+        <v>154.86261919999987</v>
       </c>
       <c r="D62" s="15">
         <f>-'M7 Financement'!D61</f>
-        <v>137.97384000000011</v>
+        <v>138.66232166400027</v>
       </c>
       <c r="E62" s="15">
         <f>-'M7 Financement'!E61</f>
-        <v>28.98583520000011</v>
+        <v>29.694971313920178</v>
       </c>
       <c r="F62" s="15">
         <f>-'M7 Financement'!F61</f>
-        <v>-26.63174974399999</v>
+        <v>-25.901339546662257</v>
       </c>
       <c r="G62" s="15">
         <f>-'M7 Financement'!G61</f>
-        <v>21.261297763679977</v>
+        <v>22.013620266937551</v>
       </c>
     </row>
     <row r="63" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B63" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="C63" s="25">
+      <c r="C63" s="26">
         <f>'M7 Financement'!C62</f>
-        <v>154.4169999999998</v>
-      </c>
-      <c r="D63" s="25">
+        <v>154.86261919999987</v>
+      </c>
+      <c r="D63" s="26">
         <f>C63+'M7 Financement'!D62</f>
-        <v>292.39083999999991</v>
-      </c>
-      <c r="E63" s="25">
+        <v>293.52494086400014</v>
+      </c>
+      <c r="E63" s="26">
         <f>D63+'M7 Financement'!E62</f>
-        <v>321.37667520000002</v>
-      </c>
-      <c r="F63" s="25">
+        <v>323.21991217792032</v>
+      </c>
+      <c r="F63" s="26">
         <f>E63+'M7 Financement'!F62</f>
-        <v>294.74492545600003</v>
-      </c>
-      <c r="G63" s="25">
+        <v>297.31857263125806</v>
+      </c>
+      <c r="G63" s="26">
         <f>F63+'M7 Financement'!G62</f>
-        <v>316.00622321968001</v>
+        <v>319.33219289819561</v>
       </c>
     </row>
     <row r="64" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B64" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="C64" s="20">
+      <c r="C64" s="21">
         <f>MAX(0,'M7 Financement'!C63)</f>
-        <v>154.4169999999998</v>
-      </c>
-      <c r="D64" s="20">
+        <v>154.86261919999987</v>
+      </c>
+      <c r="D64" s="21">
         <f>MAX(0,'M7 Financement'!D63)</f>
-        <v>292.39083999999991</v>
-      </c>
-      <c r="E64" s="20">
+        <v>293.52494086400014</v>
+      </c>
+      <c r="E64" s="21">
         <f>MAX(0,'M7 Financement'!E63)</f>
-        <v>321.37667520000002</v>
-      </c>
-      <c r="F64" s="20">
+        <v>323.21991217792032</v>
+      </c>
+      <c r="F64" s="21">
         <f>MAX(0,'M7 Financement'!F63)</f>
-        <v>294.74492545600003</v>
-      </c>
-      <c r="G64" s="20">
+        <v>297.31857263125806</v>
+      </c>
+      <c r="G64" s="21">
         <f>MAX(0,'M7 Financement'!G63)</f>
-        <v>316.00622321968001</v>
+        <v>319.33219289819561</v>
       </c>
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B65" s="8" t="s">
         <v>341</v>
       </c>
-      <c r="C65" s="26">
+      <c r="C65" s="27">
         <f>'M7 Financement'!C38</f>
-        <v>-7.1629999999999683</v>
-      </c>
-      <c r="D65" s="26">
+        <v>-6.7173808000000559</v>
+      </c>
+      <c r="D65" s="27">
         <f>'M7 Financement'!D38</f>
-        <v>12.579839999999773</v>
-      </c>
-      <c r="E65" s="26">
+        <v>13.268321664000045</v>
+      </c>
+      <c r="E65" s="27">
         <f>'M7 Financement'!E38</f>
-        <v>25.413835200000047</v>
-      </c>
-      <c r="F65" s="26">
+        <v>26.122971313920168</v>
+      </c>
+      <c r="F65" s="27">
         <f>'M7 Financement'!F38</f>
-        <v>23.368250256000142</v>
-      </c>
-      <c r="G65" s="26">
+        <v>24.098660453337665</v>
+      </c>
+      <c r="G65" s="27">
         <f>'M7 Financement'!G38</f>
-        <v>21.261297763679998</v>
+        <v>22.013620266937696</v>
       </c>
     </row>
     <row r="66" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B66" s="8" t="s">
         <v>342</v>
       </c>
-      <c r="C66" s="26">
+      <c r="C66" s="27">
         <f>'M7 Financement'!C56</f>
         <v>161.57999999999998</v>
       </c>
-      <c r="D66" s="26">
+      <c r="D66" s="27">
         <f>'M7 Financement'!D56</f>
         <v>125.39400000000001</v>
       </c>
-      <c r="E66" s="26">
+      <c r="E66" s="27">
         <f>'M7 Financement'!E56</f>
         <v>3.5719999999999987</v>
       </c>
-      <c r="F66" s="26">
+      <c r="F66" s="27">
         <f>'M7 Financement'!F56</f>
         <v>-50</v>
       </c>
-      <c r="G66" s="26">
+      <c r="G66" s="27">
         <f>'M7 Financement'!G56</f>
         <v>0</v>
       </c>
@@ -7462,25 +7464,25 @@
       <c r="B67" s="8" t="s">
         <v>343</v>
       </c>
-      <c r="C67" s="27">
+      <c r="C67" s="28">
         <f>'M7 Financement'!C62-'M7 Financement'!C38-'M7 Financement'!C56</f>
-        <v>-2.2737367544323206E-13</v>
-      </c>
-      <c r="D67" s="27">
+        <v>0</v>
+      </c>
+      <c r="D67" s="28">
         <f>'M7 Financement'!D62-'M7 Financement'!D38-'M7 Financement'!D56</f>
-        <v>3.2684965844964609E-13</v>
-      </c>
-      <c r="E67" s="27">
+        <v>2.2737367544323206E-13</v>
+      </c>
+      <c r="E67" s="28">
         <f>'M7 Financement'!E62-'M7 Financement'!E38-'M7 Financement'!E56</f>
-        <v>6.4392935428259079E-14</v>
-      </c>
-      <c r="F67" s="27">
+        <v>1.1102230246251565E-14</v>
+      </c>
+      <c r="F67" s="28">
         <f>'M7 Financement'!F62-'M7 Financement'!F38-'M7 Financement'!F56</f>
-        <v>-1.2789769243681803E-13</v>
-      </c>
-      <c r="G67" s="27">
+        <v>7.815970093361102E-14</v>
+      </c>
+      <c r="G67" s="28">
         <f>'M7 Financement'!G62-'M7 Financement'!G38-'M7 Financement'!G56</f>
-        <v>-2.1316282072803006E-14</v>
+        <v>-1.4566126083082054E-13</v>
       </c>
     </row>
     <row r="70" spans="2:7" x14ac:dyDescent="0.25">
@@ -7492,16 +7494,16 @@
       <c r="B71" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="C71" s="20">
+      <c r="C71" s="21">
         <f>MAX(C64:G64)</f>
-        <v>321.37667520000002</v>
+        <v>323.21991217792032</v>
       </c>
     </row>
     <row r="72" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B72" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="C72" s="28" t="str">
+      <c r="C72" s="29" t="str">
         <f>IF(C64='M7 Financement'!C71,"P1",IF(D64='M7 Financement'!C71,"P2",IF(E64='M7 Financement'!C71,"P3",IF(F64='M7 Financement'!C71,"P4","P5"))))</f>
         <v>P3</v>
       </c>
@@ -7520,7 +7522,7 @@
       </c>
       <c r="C74" s="15">
         <f>'M7 Financement'!G63-'M7 Financement'!F63</f>
-        <v>21.261297763679977</v>
+        <v>22.013620266937551</v>
       </c>
     </row>
     <row r="75" spans="2:7" x14ac:dyDescent="0.25">
@@ -7536,7 +7538,7 @@
       <c r="B76" s="3" t="s">
         <v>350</v>
       </c>
-      <c r="C76" s="28" t="str">
+      <c r="C76" s="29" t="str">
         <f>IF('M7 Financement'!G38&gt;0,"croissant à l'horizon",IF('M7 Financement'!G64=0,"résorbé",IF('M7 Financement'!G38=0,"plateau","non résorbé à l'horizon")))</f>
         <v>croissant à l'horizon</v>
       </c>
@@ -7545,7 +7547,7 @@
       <c r="B77" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="C77" s="29" t="s">
+      <c r="C77" s="30" t="s">
         <v>352</v>
       </c>
       <c r="D77" s="13" t="s">
@@ -7553,7 +7555,7 @@
       </c>
     </row>
     <row r="79" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="19" t="s">
+      <c r="B79" s="20" t="s">
         <v>354</v>
       </c>
     </row>
@@ -7580,7 +7582,7 @@
       </c>
     </row>
     <row r="3" spans="2:5" ht="108" x14ac:dyDescent="0.25">
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>356</v>
       </c>
     </row>
@@ -7605,7 +7607,7 @@
       <c r="C6" s="4" t="s">
         <v>360</v>
       </c>
-      <c r="D6" s="30">
+      <c r="D6" s="31">
         <f>Hypothèses!C9-Hypothèses!C6*Hypothèses!C8</f>
         <v>0</v>
       </c>
@@ -7620,7 +7622,7 @@
       <c r="C7" s="4" t="s">
         <v>362</v>
       </c>
-      <c r="D7" s="30">
+      <c r="D7" s="31">
         <f>Hypothèses!C11-Hypothèses!C10/Hypothèses!C9</f>
         <v>0</v>
       </c>
@@ -7635,7 +7637,7 @@
       <c r="C8" s="4" t="s">
         <v>363</v>
       </c>
-      <c r="D8" s="30">
+      <c r="D8" s="31">
         <f>Hypothèses!C15-1</f>
         <v>0</v>
       </c>
@@ -7650,7 +7652,7 @@
       <c r="C9" s="4" t="s">
         <v>365</v>
       </c>
-      <c r="D9" s="30">
+      <c r="D9" s="31">
         <f>'M6 Bridge'!C33-('M6 Bridge'!H6+'M6 Bridge'!H7+'M3 Stand-alone'!C15)</f>
         <v>0</v>
       </c>
@@ -7665,7 +7667,7 @@
       <c r="C10" s="4" t="s">
         <v>367</v>
       </c>
-      <c r="D10" s="30">
+      <c r="D10" s="31">
         <f>MAX(0,'M3 Stand-alone'!E11/'M3 Stand-alone'!C11-1)+MAX(0,-('M3 Stand-alone'!E11/'M3 Stand-alone'!C11))+MAX(0,'M3 Stand-alone'!F11/'M3 Stand-alone'!C11-1)+MAX(0,-('M3 Stand-alone'!F11/'M3 Stand-alone'!C11))+MAX(0,'M3 Stand-alone'!G11/'M3 Stand-alone'!C11-1)+MAX(0,-('M3 Stand-alone'!G11/'M3 Stand-alone'!C11))+MAX(0,'M3 Stand-alone'!H11/'M3 Stand-alone'!C11-1)+MAX(0,-('M3 Stand-alone'!H11/'M3 Stand-alone'!C11))+MAX(0,'M3 Stand-alone'!I11/'M3 Stand-alone'!C11-1)+MAX(0,-('M3 Stand-alone'!I11/'M3 Stand-alone'!C11))+MAX(0,'M3 Stand-alone'!E12/'M3 Stand-alone'!C12-1)+MAX(0,-('M3 Stand-alone'!E12/'M3 Stand-alone'!C12))+MAX(0,'M3 Stand-alone'!F12/'M3 Stand-alone'!C12-1)+MAX(0,-('M3 Stand-alone'!F12/'M3 Stand-alone'!C12))+MAX(0,'M3 Stand-alone'!G12/'M3 Stand-alone'!C12-1)+MAX(0,-('M3 Stand-alone'!G12/'M3 Stand-alone'!C12))+MAX(0,'M3 Stand-alone'!H12/'M3 Stand-alone'!C12-1)+MAX(0,-('M3 Stand-alone'!H12/'M3 Stand-alone'!C12))+MAX(0,'M3 Stand-alone'!I12/'M3 Stand-alone'!C12-1)+MAX(0,-('M3 Stand-alone'!I12/'M3 Stand-alone'!C12))+MAX(0,'M3 Stand-alone'!E13/'M3 Stand-alone'!C13-1)+MAX(0,-('M3 Stand-alone'!E13/'M3 Stand-alone'!C13))+MAX(0,'M3 Stand-alone'!F13/'M3 Stand-alone'!C13-1)+MAX(0,-('M3 Stand-alone'!F13/'M3 Stand-alone'!C13))+MAX(0,'M3 Stand-alone'!G13/'M3 Stand-alone'!C13-1)+MAX(0,-('M3 Stand-alone'!G13/'M3 Stand-alone'!C13))+MAX(0,'M3 Stand-alone'!H13/'M3 Stand-alone'!C13-1)+MAX(0,-('M3 Stand-alone'!H13/'M3 Stand-alone'!C13))+MAX(0,'M3 Stand-alone'!I13/'M3 Stand-alone'!C13-1)+MAX(0,-('M3 Stand-alone'!I13/'M3 Stand-alone'!C13))+MAX(0,'M3 Stand-alone'!E14/'M3 Stand-alone'!C14-1)+MAX(0,-('M3 Stand-alone'!E14/'M3 Stand-alone'!C14))+MAX(0,'M3 Stand-alone'!F14/'M3 Stand-alone'!C14-1)+MAX(0,-('M3 Stand-alone'!F14/'M3 Stand-alone'!C14))+MAX(0,'M3 Stand-alone'!G14/'M3 Stand-alone'!C14-1)+MAX(0,-('M3 Stand-alone'!G14/'M3 Stand-alone'!C14))+MAX(0,'M3 Stand-alone'!H14/'M3 Stand-alone'!C14-1)+MAX(0,-('M3 Stand-alone'!H14/'M3 Stand-alone'!C14))+MAX(0,'M3 Stand-alone'!I14/'M3 Stand-alone'!C14-1)+MAX(0,-('M3 Stand-alone'!I14/'M3 Stand-alone'!C14))</f>
         <v>0</v>
       </c>
@@ -7680,7 +7682,7 @@
       <c r="C11" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="D11" s="30">
+      <c r="D11" s="31">
         <f>('M4 TSA'!J11-('M4 TSA'!J6+'M4 TSA'!J7+'M4 TSA'!J8+'M4 TSA'!J9+'M4 TSA'!J10))+('M4 TSA'!K11-('M4 TSA'!K6+'M4 TSA'!K7+'M4 TSA'!K8+'M4 TSA'!K9+'M4 TSA'!K10))+('M4 TSA'!L11-('M4 TSA'!L6+'M4 TSA'!L7+'M4 TSA'!L8+'M4 TSA'!L9+'M4 TSA'!L10))+('M4 TSA'!M11-('M4 TSA'!M6+'M4 TSA'!M7+'M4 TSA'!M8+'M4 TSA'!M9+'M4 TSA'!M10))+('M4 TSA'!N11-('M4 TSA'!N6+'M4 TSA'!N7+'M4 TSA'!N8+'M4 TSA'!N9+'M4 TSA'!N10))</f>
         <v>0</v>
       </c>
@@ -7695,7 +7697,7 @@
       <c r="C12" s="4" t="s">
         <v>371</v>
       </c>
-      <c r="D12" s="30">
+      <c r="D12" s="31">
         <f>SUM(Calendrier!J19:J23)</f>
         <v>0</v>
       </c>
@@ -7710,7 +7712,7 @@
       <c r="C13" s="4" t="s">
         <v>373</v>
       </c>
-      <c r="D13" s="30">
+      <c r="D13" s="31">
         <f>MAX(0,-'M4 TSA'!H6)+MAX(0,'M4 TSA'!H6-'M4 TSA'!E6)+MAX(0,-'M4 TSA'!H7)+MAX(0,'M4 TSA'!H7-'M4 TSA'!E7)+MAX(0,-'M4 TSA'!H8)+MAX(0,'M4 TSA'!H8-'M4 TSA'!E8)+MAX(0,-'M4 TSA'!H9)+MAX(0,'M4 TSA'!H9-'M4 TSA'!E9)+MAX(0,-'M4 TSA'!H10)+MAX(0,'M4 TSA'!H10-'M4 TSA'!E10)</f>
         <v>0</v>
       </c>
@@ -7725,7 +7727,7 @@
       <c r="C14" s="4" t="s">
         <v>375</v>
       </c>
-      <c r="D14" s="30">
+      <c r="D14" s="31">
         <f>('M5 One-offs'!D12-('M5 One-offs'!D6+'M5 One-offs'!D7+'M5 One-offs'!D8+'M5 One-offs'!D9+'M5 One-offs'!D10+'M5 One-offs'!D11))+('M5 One-offs'!E12-('M5 One-offs'!E6+'M5 One-offs'!E7+'M5 One-offs'!E8+'M5 One-offs'!E9+'M5 One-offs'!E10+'M5 One-offs'!E11))+('M5 One-offs'!F12-('M5 One-offs'!F6+'M5 One-offs'!F7+'M5 One-offs'!F8+'M5 One-offs'!F9+'M5 One-offs'!F10+'M5 One-offs'!F11))+('M5 One-offs'!G12-('M5 One-offs'!G6+'M5 One-offs'!G7+'M5 One-offs'!G8+'M5 One-offs'!G9+'M5 One-offs'!G10+'M5 One-offs'!G11))+('M5 One-offs'!H12-('M5 One-offs'!H6+'M5 One-offs'!H7+'M5 One-offs'!H8+'M5 One-offs'!H9+'M5 One-offs'!H10+'M5 One-offs'!H11))</f>
         <v>0</v>
       </c>
@@ -7740,7 +7742,7 @@
       <c r="C15" s="4" t="s">
         <v>377</v>
       </c>
-      <c r="D15" s="30">
+      <c r="D15" s="31">
         <f>('M6 Bridge'!D31-('M6 Bridge'!D6+'M6 Bridge'!D7+'M6 Bridge'!D8+'M6 Bridge'!D9+'M6 Bridge'!D10+'M6 Bridge'!D11+'M6 Bridge'!D12+'M6 Bridge'!D13+'M6 Bridge'!D14+'M6 Bridge'!D15+'M6 Bridge'!D16+'M6 Bridge'!D17+'M6 Bridge'!D18+'M6 Bridge'!D19+'M6 Bridge'!D20+'M6 Bridge'!D21+'M6 Bridge'!D22+'M6 Bridge'!D23+'M6 Bridge'!D24+'M6 Bridge'!D25+'M6 Bridge'!D26+'M6 Bridge'!D27+'M6 Bridge'!D28+'M6 Bridge'!D29+'M6 Bridge'!D30))+('M6 Bridge'!E31-('M6 Bridge'!E6+'M6 Bridge'!E7+'M6 Bridge'!E8+'M6 Bridge'!E9+'M6 Bridge'!E10+'M6 Bridge'!E11+'M6 Bridge'!E12+'M6 Bridge'!E13+'M6 Bridge'!E14+'M6 Bridge'!E15+'M6 Bridge'!E16+'M6 Bridge'!E17+'M6 Bridge'!E18+'M6 Bridge'!E19+'M6 Bridge'!E20+'M6 Bridge'!E21+'M6 Bridge'!E22+'M6 Bridge'!E23+'M6 Bridge'!E24+'M6 Bridge'!E25+'M6 Bridge'!E26+'M6 Bridge'!E27+'M6 Bridge'!E28+'M6 Bridge'!E29+'M6 Bridge'!E30))+('M6 Bridge'!F31-('M6 Bridge'!F6+'M6 Bridge'!F7+'M6 Bridge'!F8+'M6 Bridge'!F9+'M6 Bridge'!F10+'M6 Bridge'!F11+'M6 Bridge'!F12+'M6 Bridge'!F13+'M6 Bridge'!F14+'M6 Bridge'!F15+'M6 Bridge'!F16+'M6 Bridge'!F17+'M6 Bridge'!F18+'M6 Bridge'!F19+'M6 Bridge'!F20+'M6 Bridge'!F21+'M6 Bridge'!F22+'M6 Bridge'!F23+'M6 Bridge'!F24+'M6 Bridge'!F25+'M6 Bridge'!F26+'M6 Bridge'!F27+'M6 Bridge'!F28+'M6 Bridge'!F29+'M6 Bridge'!F30))+('M6 Bridge'!G31-('M6 Bridge'!G6+'M6 Bridge'!G7+'M6 Bridge'!G8+'M6 Bridge'!G9+'M6 Bridge'!G10+'M6 Bridge'!G11+'M6 Bridge'!G12+'M6 Bridge'!G13+'M6 Bridge'!G14+'M6 Bridge'!G15+'M6 Bridge'!G16+'M6 Bridge'!G17+'M6 Bridge'!G18+'M6 Bridge'!G19+'M6 Bridge'!G20+'M6 Bridge'!G21+'M6 Bridge'!G22+'M6 Bridge'!G23+'M6 Bridge'!G24+'M6 Bridge'!G25+'M6 Bridge'!G26+'M6 Bridge'!G27+'M6 Bridge'!G28+'M6 Bridge'!G29+'M6 Bridge'!G30))+('M6 Bridge'!H31-('M6 Bridge'!H6+'M6 Bridge'!H7+'M6 Bridge'!H8+'M6 Bridge'!H9+'M6 Bridge'!H10+'M6 Bridge'!H11+'M6 Bridge'!H12+'M6 Bridge'!H13+'M6 Bridge'!H14+'M6 Bridge'!H15+'M6 Bridge'!H16+'M6 Bridge'!H17+'M6 Bridge'!H18+'M6 Bridge'!H19+'M6 Bridge'!H20+'M6 Bridge'!H21+'M6 Bridge'!H22+'M6 Bridge'!H23+'M6 Bridge'!H24+'M6 Bridge'!H25+'M6 Bridge'!H26+'M6 Bridge'!H27+'M6 Bridge'!H28+'M6 Bridge'!H29+'M6 Bridge'!H30))</f>
         <v>0</v>
       </c>
@@ -7755,7 +7757,7 @@
       <c r="C16" s="4" t="s">
         <v>379</v>
       </c>
-      <c r="D16" s="30">
+      <c r="D16" s="31">
         <f>('M7 Financement'!C15-('M7 Financement'!C10+'M7 Financement'!C11+'M7 Financement'!C12+'M7 Financement'!C13+'M7 Financement'!C14))+('M7 Financement'!D15-('M7 Financement'!D10+'M7 Financement'!D11+'M7 Financement'!D12+'M7 Financement'!D13+'M7 Financement'!D14))+('M7 Financement'!E15-('M7 Financement'!E10+'M7 Financement'!E11+'M7 Financement'!E12+'M7 Financement'!E13+'M7 Financement'!E14))+('M7 Financement'!F15-('M7 Financement'!F10+'M7 Financement'!F11+'M7 Financement'!F12+'M7 Financement'!F13+'M7 Financement'!F14))+('M7 Financement'!G15-('M7 Financement'!G10+'M7 Financement'!G11+'M7 Financement'!G12+'M7 Financement'!G13+'M7 Financement'!G14))</f>
         <v>0</v>
       </c>
@@ -7770,7 +7772,7 @@
       <c r="C17" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="D17" s="30">
+      <c r="D17" s="31">
         <f>('M7 Financement'!C62+'M7 Financement'!C61)+('M7 Financement'!D62+'M7 Financement'!D61)+('M7 Financement'!E62+'M7 Financement'!E61)+('M7 Financement'!F62+'M7 Financement'!F61)+('M7 Financement'!G62+'M7 Financement'!G61)+('M7 Financement'!C63-0-'M7 Financement'!C62)+('M7 Financement'!C64-MAX(0,'M7 Financement'!C63))+('M7 Financement'!D63-'M7 Financement'!C63-'M7 Financement'!D62)+('M7 Financement'!D64-MAX(0,'M7 Financement'!D63))+('M7 Financement'!E63-'M7 Financement'!D63-'M7 Financement'!E62)+('M7 Financement'!E64-MAX(0,'M7 Financement'!E63))+('M7 Financement'!F63-'M7 Financement'!E63-'M7 Financement'!F62)+('M7 Financement'!F64-MAX(0,'M7 Financement'!F63))+('M7 Financement'!G63-'M7 Financement'!F63-'M7 Financement'!G62)+('M7 Financement'!G64-MAX(0,'M7 Financement'!G63))</f>
         <v>0</v>
       </c>
@@ -7785,7 +7787,7 @@
       <c r="C18" s="4" t="s">
         <v>384</v>
       </c>
-      <c r="D18" s="30">
+      <c r="D18" s="31">
         <f>MAX(0,-'M7 Financement'!C64)+MAX(0,-'M7 Financement'!D64)+MAX(0,-'M7 Financement'!E64)+MAX(0,-'M7 Financement'!F64)+MAX(0,-'M7 Financement'!G64)+('M7 Financement'!C71-MAX('M7 Financement'!C64:G64))</f>
         <v>0</v>
       </c>
@@ -7856,9 +7858,9 @@
       <c r="C23" s="4" t="s">
         <v>395</v>
       </c>
-      <c r="D23" s="30">
+      <c r="D23" s="31">
         <f>SUM('M7 Financement'!C67:G67)</f>
-        <v>1.4654943925052066E-14</v>
+        <v>1.7097434579227411E-13</v>
       </c>
       <c r="E23" s="8" t="s">
         <v>382</v>
@@ -7913,7 +7915,7 @@
       <c r="C27" s="4" t="s">
         <v>403</v>
       </c>
-      <c r="D27" s="30">
+      <c r="D27" s="31">
         <f>'M6 Bridge'!C34+('M4 TSA'!J11+'M5 One-offs'!D12+'M6 Bridge'!D23+'M4 TSA'!K11+'M5 One-offs'!E12+'M6 Bridge'!E23+'M4 TSA'!L11+'M5 One-offs'!F12+'M6 Bridge'!F23+'M4 TSA'!M11+'M5 One-offs'!G12+'M6 Bridge'!G23+'M4 TSA'!N11+'M5 One-offs'!H12+'M6 Bridge'!H23)</f>
         <v>0</v>
       </c>

</xml_diff>